<commit_message>
[feat][paper] 论文第五章调整，按照Implementation, Upgrade efficiency, Upgrade Consistency, Execution Efficiency, functional Validation展开
</commit_message>
<xml_diff>
--- a/paper/image/experiments_result.xlsx
+++ b/paper/image/experiments_result.xlsx
@@ -7913,118 +7913,118 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="16.6640625" style="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.109375" style="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.6640625" style="12" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="11">
-        <v>152364</v>
-      </c>
-      <c r="C2" s="11">
-        <v>90309</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="11">
-        <v>863044</v>
-      </c>
-      <c r="C3" s="11">
-        <v>130661</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="11">
-        <v>129120</v>
-      </c>
-      <c r="C4" s="11">
-        <v>856731</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="11">
-        <v>909316</v>
-      </c>
-      <c r="C5" s="11">
-        <v>388984</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="11">
-        <v>500800</v>
-      </c>
-      <c r="C6" s="11">
-        <v>590802</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="11">
-        <v>1142620</v>
-      </c>
-      <c r="C7" s="11">
-        <v>721410</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="11">
-        <v>1144072</v>
-      </c>
-      <c r="C8" s="11">
-        <v>967127</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" s="11">
-        <v>118240</v>
-      </c>
-      <c r="C9" s="11">
-        <v>270187</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0300-000000000000}">
+  <ns0:dimension ref="A1:C9"/>
+  <ns0:sheetFormatPr defaultRowHeight="13.8" ns3:dyDescent="0.25"/>
+  <ns0:cols>
+    <ns0:col min="1" max="1" width="16.6640625" style="12" bestFit="1" customWidth="1"/>
+    <ns0:col min="2" max="2" width="19.109375" style="12" bestFit="1" customWidth="1"/>
+    <ns0:col min="3" max="3" width="17.6640625" style="12" bestFit="1" customWidth="1"/>
+  </ns0:cols>
+  <ns0:sheetData>
+    <ns0:row r="1" spans="1:3" ns3:dyDescent="0.25">
+      <ns0:c r="A1" s="3" t="s">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="B1" s="10" t="s">
+        <ns0:v>77</ns0:v>
+      </ns0:c>
+      <ns0:c r="C1" s="10" t="s">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="2" spans="1:3" ns3:dyDescent="0.25">
+      <ns0:c r="A2" s="4" t="s">
+        <ns0:v>2</ns0:v>
+      </ns0:c>
+      <ns0:c r="B2" s="11" t="n">
+        <ns0:v>154268</ns0:v>
+      </ns0:c>
+      <ns0:c r="C2" s="11" t="n">
+        <ns0:v>90309</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="3" spans="1:3" ns3:dyDescent="0.25">
+      <ns0:c r="A3" s="4" t="s">
+        <ns0:v>3</ns0:v>
+      </ns0:c>
+      <ns0:c r="B3" s="11" t="n">
+        <ns0:v>128168</ns0:v>
+      </ns0:c>
+      <ns0:c r="C3" s="11" t="n">
+        <ns0:v>130661</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="4" spans="1:3" ns3:dyDescent="0.25">
+      <ns0:c r="A4" s="4" t="s">
+        <ns0:v>4</ns0:v>
+      </ns0:c>
+      <ns0:c r="B4" s="11" t="n">
+        <ns0:v>130860</ns0:v>
+      </ns0:c>
+      <ns0:c r="C4" s="11" t="n">
+        <ns0:v>856731</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="5" spans="1:3" ns3:dyDescent="0.25">
+      <ns0:c r="A5" s="4" t="s">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+      <ns0:c r="B5" s="11" t="n">
+        <ns0:v>175668</ns0:v>
+      </ns0:c>
+      <ns0:c r="C5" s="11" t="n">
+        <ns0:v>388984</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="6" spans="1:3" ns3:dyDescent="0.25">
+      <ns0:c r="A6" s="4" t="s">
+        <ns0:v>6</ns0:v>
+      </ns0:c>
+      <ns0:c r="B6" s="11" t="n">
+        <ns0:v>503168</ns0:v>
+      </ns0:c>
+      <ns0:c r="C6" s="11" t="n">
+        <ns0:v>590802</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="7" spans="1:3" ns3:dyDescent="0.25">
+      <ns0:c r="A7" s="4" t="s">
+        <ns0:v>7</ns0:v>
+      </ns0:c>
+      <ns0:c r="B7" s="11" t="n">
+        <ns0:v>528744</ns0:v>
+      </ns0:c>
+      <ns0:c r="C7" s="11" t="n">
+        <ns0:v>721410</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="8" spans="1:3" ns3:dyDescent="0.25">
+      <ns0:c r="A8" s="4" t="s">
+        <ns0:v>8</ns0:v>
+      </ns0:c>
+      <ns0:c r="B8" s="11" t="n">
+        <ns0:v>531232</ns0:v>
+      </ns0:c>
+      <ns0:c r="C8" s="11" t="n">
+        <ns0:v>967127</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="9" spans="1:3" ns3:dyDescent="0.25">
+      <ns0:c r="A9" s="4" t="s">
+        <ns0:v>9</ns0:v>
+      </ns0:c>
+      <ns0:c r="B9" s="11" t="n">
+        <ns0:v>120372</ns0:v>
+      </ns0:c>
+      <ns0:c r="C9" s="11" t="n">
+        <ns0:v>270187</ns0:v>
+      </ns0:c>
+    </ns0:row>
+  </ns0:sheetData>
+  <ns0:phoneticPr fontId="3" type="noConversion"/>
+  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</ns0:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>